<commit_message>
Finished up convergence, cleaned up code
</commit_message>
<xml_diff>
--- a/docs/RAW_DATA.xlsx
+++ b/docs/RAW_DATA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Github\sp-lt-pv\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA62813-DAEC-4EA2-ACCE-D4A20E0B11B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D28EC25-588E-4FEA-AB8D-FBCAD4B9D8C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -172,9 +172,6 @@
     <t>ZMesh_Y</t>
   </si>
   <si>
-    <t>Z Mesh_t</t>
-  </si>
-  <si>
     <t>AM15Flat_Y</t>
   </si>
   <si>
@@ -203,6 +200,9 @@
   </si>
   <si>
     <t>AM15_X</t>
+  </si>
+  <si>
+    <t>ZMesh_t</t>
   </si>
 </sst>
 </file>
@@ -739,34 +739,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" t="s">
         <v>48</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>49</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>50</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" t="s">
         <v>51</v>
       </c>
-      <c r="F1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>52</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>53</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>54</v>
-      </c>
-      <c r="J1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
@@ -7354,7 +7354,7 @@
         <v>46</v>
       </c>
       <c r="L1" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
@@ -7593,7 +7593,7 @@
         <v>268.88099999999997</v>
       </c>
       <c r="I8">
-        <v>5320</v>
+        <v>1872</v>
       </c>
       <c r="J8" s="1">
         <v>10</v>

</xml_diff>